<commit_message>
Added family booking flow
</commit_message>
<xml_diff>
--- a/src/test/resources/BooKIngResistratinData.xlsx
+++ b/src/test/resources/BooKIngResistratinData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ravibhushan.Kumar\eclipse-workspace\Project_SAUDIA\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CFE57D2-A67C-4D22-98F1-BF3BD298723B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC75D8DC-6C8F-435E-8E19-24EA8519B83D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="14040" xr2:uid="{95A23CBA-6176-416D-B3C6-85753400ABEE}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="117">
   <si>
     <t>TestCaseID</t>
   </si>
@@ -111,9 +111,6 @@
     <t>md.nazir@quadlabs.com</t>
   </si>
   <si>
-    <t>8454963279</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 50-249 </t>
   </si>
   <si>
@@ -273,9 +270,6 @@
     <t>Prince</t>
   </si>
   <si>
-    <t>7896541236</t>
-  </si>
-  <si>
     <t>Department_Name</t>
   </si>
   <si>
@@ -360,18 +354,9 @@
     <t>Mr.</t>
   </si>
   <si>
-    <t>Ramesh</t>
-  </si>
-  <si>
-    <t>Mishra</t>
-  </si>
-  <si>
     <t>Male</t>
   </si>
   <si>
-    <t>EMP012</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Administrator</t>
   </si>
   <si>
@@ -382,6 +367,18 @@
   </si>
   <si>
     <t>Password</t>
+  </si>
+  <si>
+    <t>Sharma</t>
+  </si>
+  <si>
+    <t>Suresh</t>
+  </si>
+  <si>
+    <t>8789395155</t>
+  </si>
+  <si>
+    <t>EMP0124</t>
   </si>
 </sst>
 </file>
@@ -872,139 +869,139 @@
         <v>17</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="S1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="U1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="V1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="X1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="U1" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="V1" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="W1" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="X1" s="1" t="s">
-        <v>41</v>
-      </c>
       <c r="Y1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="Z1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="Z1" s="1" t="s">
-        <v>46</v>
-      </c>
       <c r="AA1" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="AB1" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="AC1" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="AC1" s="1" t="s">
-        <v>51</v>
-      </c>
       <c r="AD1" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="AE1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="AF1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="AF1" s="1" t="s">
+      <c r="AG1" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="AG1" s="1" t="s">
-        <v>58</v>
-      </c>
       <c r="AH1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="AI1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="AJ1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="AK1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="AL1" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="AI1" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="AJ1" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="AK1" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="AL1" s="1" t="s">
-        <v>61</v>
-      </c>
       <c r="AM1" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="AN1" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="AN1" s="1" t="s">
+      <c r="AO1" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="AO1" s="1" t="s">
+      <c r="AP1" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="AP1" s="1" t="s">
+      <c r="AQ1" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="AQ1" s="1" t="s">
-        <v>77</v>
-      </c>
       <c r="AR1" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="AS1" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="AS1" s="1" t="s">
+      <c r="AT1" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="AT1" s="1" t="s">
-        <v>86</v>
-      </c>
       <c r="AU1" s="1" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="AV1" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="AW1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="AW1" s="1" t="s">
+      <c r="AX1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="AX1" s="1" t="s">
+      <c r="AY1" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="AZ1" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="BA1" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="AY1" s="1" t="s">
+      <c r="BB1" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="BC1" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="AZ1" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="BA1" s="1" t="s">
+      <c r="BD1" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="BB1" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="BC1" s="1" t="s">
+      <c r="BE1" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="BD1" s="1" t="s">
+      <c r="BF1" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="BE1" s="1" t="s">
+      <c r="BG1" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="BF1" s="1" t="s">
+      <c r="BH1" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="BG1" s="1" t="s">
+      <c r="BI1" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="BH1" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="BI1" s="1" t="s">
-        <v>103</v>
-      </c>
       <c r="BJ1" s="1" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
     </row>
     <row r="2" spans="1:62" x14ac:dyDescent="0.25">
@@ -1015,13 +1012,13 @@
         <v>11</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>19</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>20</v>
@@ -1048,151 +1045,151 @@
         <v>26</v>
       </c>
       <c r="N2" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="O2" s="1">
+        <v>4558975460</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="R2" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="S2" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="O2" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="P2" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q2" s="1" t="s">
+      <c r="T2" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="R2" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="S2" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="T2" s="1" t="s">
-        <v>30</v>
       </c>
       <c r="U2" s="1" t="s">
         <v>26</v>
       </c>
       <c r="V2" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="W2" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="X2" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="W2" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="X2" s="1" t="s">
-        <v>43</v>
-      </c>
       <c r="Y2" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="Z2" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="Z2" s="1" t="s">
+      <c r="AA2" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="AA2" s="1" t="s">
-        <v>49</v>
-      </c>
       <c r="AB2" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="AC2" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="AC2" s="1" t="s">
-        <v>53</v>
-      </c>
       <c r="AD2" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="AE2" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="AF2" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="AF2" s="1" t="s">
+      <c r="AG2" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="AH2" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="AG2" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="AH2" s="1" t="s">
-        <v>71</v>
-      </c>
       <c r="AI2" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AJ2" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="AK2" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="AL2" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AM2" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="AN2" t="s">
         <v>78</v>
       </c>
-      <c r="AN2" t="s">
+      <c r="AO2" t="s">
         <v>79</v>
-      </c>
-      <c r="AO2" t="s">
-        <v>80</v>
       </c>
       <c r="AP2" s="2" t="s">
         <v>26</v>
       </c>
       <c r="AQ2" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="AR2" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="AR2" s="1" t="s">
+      <c r="AS2" t="s">
         <v>83</v>
       </c>
-      <c r="AS2" t="s">
-        <v>85</v>
-      </c>
       <c r="AT2" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="AU2" t="s">
+        <v>87</v>
+      </c>
+      <c r="AV2" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="AV2" s="1" t="s">
+      <c r="AW2" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="AW2" s="1" t="s">
-        <v>93</v>
-      </c>
       <c r="AX2" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="AY2" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="AZ2" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="BA2" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="BB2" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="AY2" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="AZ2" s="1" t="s">
+      <c r="BC2" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="BA2" s="1" t="s">
+      <c r="BD2" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="BE2" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="BF2" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="BG2" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="BB2" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="BC2" s="1" t="s">
+      <c r="BH2" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="BI2" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="BD2" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="BE2" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="BF2" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="BG2" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="BH2" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="BI2" s="1" t="s">
-        <v>114</v>
-      </c>
       <c r="BJ2" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:62" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Updated flight booking automation and family trip flow
</commit_message>
<xml_diff>
--- a/src/test/resources/BooKIngResistratinData.xlsx
+++ b/src/test/resources/BooKIngResistratinData.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ravibhushan.Kumar\eclipse-workspace\Project_SAUDIA\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC75D8DC-6C8F-435E-8E19-24EA8519B83D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CB6B5E1-0D22-4C62-B215-C944BB8BDCA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="14040" xr2:uid="{95A23CBA-6176-416D-B3C6-85753400ABEE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11160" xr2:uid="{95A23CBA-6176-416D-B3C6-85753400ABEE}"/>
   </bookViews>
   <sheets>
     <sheet name="BookingRegistrationdata" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="149">
   <si>
     <t>TestCaseID</t>
   </si>
@@ -63,9 +64,6 @@
     <t>TC01</t>
   </si>
   <si>
-    <t>Verify User is able to create Registartion for booking</t>
-  </si>
-  <si>
     <t>Industry</t>
   </si>
   <si>
@@ -93,18 +91,9 @@
     <t>8523697410</t>
   </si>
   <si>
-    <t>India</t>
-  </si>
-  <si>
-    <t>Delhi</t>
-  </si>
-  <si>
     <t>122018</t>
   </si>
   <si>
-    <t>240</t>
-  </si>
-  <si>
     <t>Sohna road</t>
   </si>
   <si>
@@ -126,9 +115,6 @@
     <t>English</t>
   </si>
   <si>
-    <t xml:space="preserve">+91 </t>
-  </si>
-  <si>
     <t>Add new</t>
   </si>
   <si>
@@ -237,155 +223,266 @@
     <t xml:space="preserve">  Credit Card </t>
   </si>
   <si>
-    <t xml:space="preserve"> VISA</t>
+    <t>GTM5253618070</t>
+  </si>
+  <si>
+    <t>Businessunit_code</t>
+  </si>
+  <si>
+    <t>Business_Unit_name</t>
+  </si>
+  <si>
+    <t>Business_unit_Manager</t>
+  </si>
+  <si>
+    <t>Business_unit_mail</t>
+  </si>
+  <si>
+    <t>Business_unit_ContactNumber</t>
+  </si>
+  <si>
+    <t>QL01</t>
+  </si>
+  <si>
+    <t>Flight Booking</t>
+  </si>
+  <si>
+    <t>Prince</t>
+  </si>
+  <si>
+    <t>Department_Name</t>
+  </si>
+  <si>
+    <t>Testing</t>
+  </si>
+  <si>
+    <t>Designation</t>
+  </si>
+  <si>
+    <t>Software Test Engineer</t>
+  </si>
+  <si>
+    <t>CategoryName</t>
+  </si>
+  <si>
+    <t>CategoryCode</t>
+  </si>
+  <si>
+    <t>Automation</t>
+  </si>
+  <si>
+    <t>QAA</t>
+  </si>
+  <si>
+    <t>TravelCategory</t>
+  </si>
+  <si>
+    <t>Business</t>
+  </si>
+  <si>
+    <t>TripType</t>
+  </si>
+  <si>
+    <t>Business Trip</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nationality </t>
+  </si>
+  <si>
+    <t xml:space="preserve">PlaceofResidence </t>
+  </si>
+  <si>
+    <t>DOB</t>
+  </si>
+  <si>
+    <t>Title</t>
+  </si>
+  <si>
+    <t>FirstName</t>
+  </si>
+  <si>
+    <t>Lastname</t>
+  </si>
+  <si>
+    <t>Gender</t>
+  </si>
+  <si>
+    <t>EmployeeNumber</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>UserType</t>
+  </si>
+  <si>
+    <t>Passport</t>
+  </si>
+  <si>
+    <t>PassportExpiryDate</t>
+  </si>
+  <si>
+    <t>Password</t>
+  </si>
+  <si>
+    <t>8789395155</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Saudi Arabia </t>
+  </si>
+  <si>
+    <t>Agraa</t>
+  </si>
+  <si>
+    <t>Dhahran</t>
+  </si>
+  <si>
+    <t>2403</t>
+  </si>
+  <si>
+    <t>+966</t>
+  </si>
+  <si>
+    <t>Verify User is able to Update  company Details in Company Profile</t>
+  </si>
+  <si>
+    <t>TC02</t>
+  </si>
+  <si>
+    <t>Verify User is able to Update  Cost Centre in Company Profile</t>
+  </si>
+  <si>
+    <t>TC03</t>
+  </si>
+  <si>
+    <t>TC04</t>
+  </si>
+  <si>
+    <t>Verify User is able to Update Project in Company Profile</t>
+  </si>
+  <si>
+    <t>TC05</t>
+  </si>
+  <si>
+    <t>Verify User is able to Add credit card in Company Profile</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> VISA </t>
   </si>
   <si>
     <t>4111-1111-1111-1111</t>
   </si>
   <si>
-    <t>GTM5253618070</t>
-  </si>
-  <si>
-    <t>Businessunit_code</t>
-  </si>
-  <si>
-    <t>Business_Unit_name</t>
-  </si>
-  <si>
-    <t>Business_unit_Manager</t>
-  </si>
-  <si>
-    <t>Business_unit_mail</t>
-  </si>
-  <si>
-    <t>Business_unit_ContactNumber</t>
-  </si>
-  <si>
-    <t>QL01</t>
-  </si>
-  <si>
-    <t>Flight Booking</t>
-  </si>
-  <si>
-    <t>Prince</t>
-  </si>
-  <si>
-    <t>Department_Name</t>
-  </si>
-  <si>
-    <t>Testing</t>
-  </si>
-  <si>
-    <t>Designation</t>
-  </si>
-  <si>
-    <t>Software Test Engineer</t>
-  </si>
-  <si>
-    <t>CategoryName</t>
-  </si>
-  <si>
-    <t>CategoryCode</t>
-  </si>
-  <si>
-    <t>Automation</t>
-  </si>
-  <si>
-    <t>QAA</t>
-  </si>
-  <si>
-    <t>TravelCategory</t>
-  </si>
-  <si>
-    <t>Business</t>
-  </si>
-  <si>
-    <t>TripType</t>
-  </si>
-  <si>
-    <t>Business Trip</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nationality </t>
-  </si>
-  <si>
-    <t xml:space="preserve">PlaceofResidence </t>
-  </si>
-  <si>
-    <t>DOB</t>
-  </si>
-  <si>
-    <t>Title</t>
-  </si>
-  <si>
-    <t>FirstName</t>
-  </si>
-  <si>
-    <t>Lastname</t>
-  </si>
-  <si>
-    <t>Gender</t>
-  </si>
-  <si>
-    <t>EmployeeNumber</t>
-  </si>
-  <si>
-    <t>Email</t>
-  </si>
-  <si>
-    <t>UserType</t>
-  </si>
-  <si>
-    <t>Passport</t>
-  </si>
-  <si>
-    <t>PassportExpiryDate</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> India </t>
-  </si>
-  <si>
-    <t>PASS4562</t>
-  </si>
-  <si>
-    <t>10-Feb-2036</t>
-  </si>
-  <si>
-    <t>Mr.</t>
-  </si>
-  <si>
-    <t>Male</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Administrator</t>
-  </si>
-  <si>
-    <t>rsbhushan@gmail.com</t>
-  </si>
-  <si>
-    <t>10-Feb-1991</t>
-  </si>
-  <si>
-    <t>Password</t>
+    <t>TC06</t>
+  </si>
+  <si>
+    <t>Verify User is able to Update  Businessunit in Company Profile</t>
+  </si>
+  <si>
+    <t>TC07</t>
+  </si>
+  <si>
+    <t>Verify User is able to Update  Travel Profile</t>
+  </si>
+  <si>
+    <t>Verify User is able to Add  Office Location in Company Profile</t>
+  </si>
+  <si>
+    <t>TC08</t>
+  </si>
+  <si>
+    <t>TC09</t>
+  </si>
+  <si>
+    <t>Edit</t>
+  </si>
+  <si>
+    <t>delete</t>
+  </si>
+  <si>
+    <t>Verify User is able to Delete Office Location in Company Profile</t>
+  </si>
+  <si>
+    <t>Verify User is able to Edit  Office Location in Company Profile</t>
+  </si>
+  <si>
+    <t>MTG Corporate</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 110097</t>
+  </si>
+  <si>
+    <t>7878452423</t>
+  </si>
+  <si>
+    <t>Jubail</t>
+  </si>
+  <si>
+    <t>Verify User is able to Add  Cost Centre in Company Profile</t>
+  </si>
+  <si>
+    <t>TC10</t>
   </si>
   <si>
     <t>Sharma</t>
   </si>
   <si>
-    <t>Suresh</t>
-  </si>
-  <si>
-    <t>8789395155</t>
-  </si>
-  <si>
-    <t>EMP0124</t>
+    <t>S01</t>
+  </si>
+  <si>
+    <t>Verify User is able to Delete  Cost Centre in Company Profile</t>
+  </si>
+  <si>
+    <t>TC11</t>
+  </si>
+  <si>
+    <t>Verify User is able to Add Office Location in Company Profile</t>
+  </si>
+  <si>
+    <t>Verify User is able to Delete  Office Location in Company Profile</t>
+  </si>
+  <si>
+    <t>Verify User is able to Add  Project in Company Profile</t>
+  </si>
+  <si>
+    <t>TC12</t>
+  </si>
+  <si>
+    <t>TC13</t>
+  </si>
+  <si>
+    <t>TS002</t>
+  </si>
+  <si>
+    <t>Verify User is able to Delete  Project in Company Profile</t>
+  </si>
+  <si>
+    <t>Verify User is able to Update  Project in Company Profile</t>
+  </si>
+  <si>
+    <t>Verify User is able to Add  Businessunit in Company Profile</t>
+  </si>
+  <si>
+    <t>Verify User is able to Delete  Businessunit in Company Profile</t>
+  </si>
+  <si>
+    <t>8789395157</t>
+  </si>
+  <si>
+    <t>rsbhushan67@gmail.com</t>
+  </si>
+  <si>
+    <t>TC14</t>
+  </si>
+  <si>
+    <t>TC15</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -397,6 +494,12 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -762,7 +865,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3701056F-C09A-4200-A54F-A616771A587D}">
-  <dimension ref="A1:BJ3"/>
+  <dimension ref="A1:BJ16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.7109375" customWidth="1"/>
@@ -770,6 +873,7 @@
     <col min="4" max="4" width="21.140625" customWidth="1"/>
     <col min="5" max="5" width="24.42578125" customWidth="1"/>
     <col min="6" max="6" width="23.42578125" customWidth="1"/>
+    <col min="7" max="7" width="14.5703125" customWidth="1"/>
     <col min="10" max="10" width="16.140625" customWidth="1"/>
     <col min="11" max="11" width="18" customWidth="1"/>
     <col min="12" max="12" width="15.28515625" customWidth="1"/>
@@ -789,7 +893,7 @@
     <col min="29" max="29" width="14.42578125" customWidth="1"/>
     <col min="30" max="30" width="14.28515625" customWidth="1"/>
     <col min="31" max="31" width="16.140625" customWidth="1"/>
-    <col min="32" max="32" width="14.85546875" customWidth="1"/>
+    <col min="32" max="32" width="24.5703125" customWidth="1"/>
     <col min="33" max="33" width="21.7109375" customWidth="1"/>
     <col min="34" max="34" width="33.28515625" customWidth="1"/>
     <col min="35" max="35" width="17.140625" customWidth="1"/>
@@ -824,16 +928,16 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>13</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>14</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>2</v>
@@ -851,10 +955,10 @@
         <v>6</v>
       </c>
       <c r="L1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="M1" s="1" t="s">
         <v>15</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>16</v>
       </c>
       <c r="N1" s="1" t="s">
         <v>7</v>
@@ -866,142 +970,142 @@
         <v>9</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="R1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="U1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="S1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="T1" s="1" t="s">
+      <c r="V1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="U1" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="V1" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="W1" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="X1" s="1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="AA1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="AA1" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="AB1" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AD1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="AE1" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="AD1" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="AE1" s="1" t="s">
+      <c r="AF1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="AG1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="AH1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AI1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="AJ1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="AK1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="AL1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="AF1" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="AG1" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="AH1" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="AI1" s="1" t="s">
+      <c r="AM1" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="AJ1" s="1" t="s">
+      <c r="AN1" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="AK1" s="1" t="s">
+      <c r="AO1" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="AL1" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="AM1" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="AN1" s="1" t="s">
+      <c r="AP1" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="AQ1" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="AR1" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="AO1" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="AP1" s="1" t="s">
+      <c r="AS1" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="AQ1" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="AR1" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="AS1" s="1" t="s">
-        <v>82</v>
-      </c>
       <c r="AT1" s="1" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="AU1" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="AV1" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="AW1" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="AX1" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="AV1" s="1" t="s">
+      <c r="AY1" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="AZ1" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="BA1" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="BB1" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="BC1" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="AW1" s="1" t="s">
+      <c r="BD1" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="BE1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="AX1" s="1" t="s">
+      <c r="BF1" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="BG1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="AY1" s="1" t="s">
+      <c r="BH1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="AZ1" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="BA1" s="1" t="s">
+      <c r="BI1" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="BB1" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="BC1" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="BD1" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="BE1" s="1" t="s">
+      <c r="BJ1" s="1" t="s">
         <v>97</v>
-      </c>
-      <c r="BF1" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="BG1" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="BH1" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="BI1" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="BJ1" s="1" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="2" spans="1:62" x14ac:dyDescent="0.25">
@@ -1009,197 +1113,739 @@
         <v>10</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>11</v>
+        <v>104</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="D2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="J2" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="K2" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="L2" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="M2" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="I2" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>26</v>
-      </c>
       <c r="N2" s="1" t="s">
-        <v>32</v>
+        <v>103</v>
       </c>
       <c r="O2" s="1">
         <v>4558975460</v>
       </c>
       <c r="P2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="R2" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="Q2" s="1" t="s">
+      <c r="S2" s="1"/>
+      <c r="T2" s="1"/>
+      <c r="U2" s="1"/>
+      <c r="V2" s="1"/>
+      <c r="W2" s="1"/>
+      <c r="X2" s="1"/>
+      <c r="AA2" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="AM2" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="3" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>105</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="S3" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="T3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="U3" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="V3" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="W3" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="X3" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>107</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="L4" s="1"/>
+      <c r="S4" s="1" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="5" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>108</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="S5" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="R2" s="1" t="s">
-        <v>31</v>
+      <c r="T5" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="U5" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="V5" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="W5" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="X5" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="6" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="S6" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y6" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="Z6" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="7" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>114</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="S7" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="Y7" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="Z7" s="1" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="8" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>116</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="S8" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="Y8" s="1"/>
+      <c r="Z8" s="1"/>
+    </row>
+    <row r="9" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>119</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="S9" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="AB9" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="AC9" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="10" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>120</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="S10" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="AB10" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="AC10" s="1" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="11" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>130</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="S11" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="AB11" s="1"/>
+      <c r="AC11" s="1"/>
+    </row>
+    <row r="12" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>134</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="S12" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="AD12" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="AE12" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="AF12" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="AG12" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="AH12" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="AI12" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="AJ12" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="AK12" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="AL12" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="13" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>138</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="S13" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="AN13" t="s">
+        <v>71</v>
+      </c>
+      <c r="AO13" t="s">
+        <v>72</v>
+      </c>
+      <c r="AP13" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="AQ13" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="14" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>139</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="S14" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="AN14" t="s">
+        <v>71</v>
+      </c>
+      <c r="AO14" t="s">
+        <v>72</v>
+      </c>
+      <c r="AP14" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="AQ14" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="15" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>147</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="S15" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="AP15" s="2"/>
+      <c r="AQ15" s="1"/>
+    </row>
+    <row r="16" spans="1:62" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>148</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="AR16" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="AS16" t="s">
+        <v>76</v>
+      </c>
+      <c r="AT16" t="s">
+        <v>79</v>
+      </c>
+      <c r="AU16" t="s">
+        <v>80</v>
+      </c>
+      <c r="AV16" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="AW16" s="1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="AP13" r:id="rId1" xr:uid="{75D3A9FE-85AB-4F9C-97DC-42F495760BA0}"/>
+    <hyperlink ref="AP14" r:id="rId2" xr:uid="{ABCF4F25-17C1-40EA-A253-4ADA44730EC6}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC518EC1-753A-405F-8500-A86E99DEEBE8}">
+  <dimension ref="A1:AW16"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="O1" s="1">
+        <v>4558975460</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="1"/>
+      <c r="T1" s="1"/>
+      <c r="U1" s="1"/>
+      <c r="V1" s="1"/>
+      <c r="W1" s="1"/>
+      <c r="X1" s="1"/>
+      <c r="AA1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="AM1" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>21</v>
       </c>
       <c r="S2" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="T2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="U2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="V2" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="W2" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="T2" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="U2" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="V2" s="1" t="s">
+      <c r="X2" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>107</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="L3" s="1"/>
+      <c r="S3" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="T3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="U3" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="V3" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="W3" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="X3" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>108</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="L4" s="1"/>
+      <c r="S4" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="T4" s="1"/>
+      <c r="U4" s="1"/>
+      <c r="V4" s="1"/>
+      <c r="W4" s="1"/>
+      <c r="X4" s="1"/>
+    </row>
+    <row r="5" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>110</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="Y5" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="W2" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="X2" s="1" t="s">
+      <c r="Z5" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="Y2" s="1" t="s">
+    </row>
+    <row r="6" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>114</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="AB6" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="Z2" s="1" t="s">
+      <c r="AC6" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="AA2" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="AB2" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="AC2" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="AD2" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="AE2" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="AF2" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="AG2" s="1" t="s">
+    </row>
+    <row r="7" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>116</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD7" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="AE7" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="AF7" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="AG7" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="AH7" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="AI7" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="AJ7" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="AH2" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="AI2" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="AJ2" s="1" t="s">
+      <c r="AK7" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="AL7" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="8" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>119</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="AN8" t="s">
+        <v>71</v>
+      </c>
+      <c r="AO8" t="s">
+        <v>72</v>
+      </c>
+      <c r="AP8" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="AQ8" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="9" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>120</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="AR9" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="AS9" t="s">
+        <v>76</v>
+      </c>
+      <c r="AT9" t="s">
+        <v>79</v>
+      </c>
+      <c r="AU9" t="s">
+        <v>80</v>
+      </c>
+      <c r="AV9" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="AW9" s="1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="12" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>110</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="Y12" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="Z12" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="13" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>114</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="AB13" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="AC13" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="14" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>116</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD14" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="AE14" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="AK2" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="AL2" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="AM2" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="AN2" t="s">
-        <v>78</v>
-      </c>
-      <c r="AO2" t="s">
+      <c r="AF14" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="AG14" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="AH14" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="AI14" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="AJ14" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="AK14" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="AL14" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="15" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>119</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="AN15" t="s">
+        <v>71</v>
+      </c>
+      <c r="AO15" t="s">
+        <v>72</v>
+      </c>
+      <c r="AP15" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="AQ15" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="16" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>120</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="AR16" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="AS16" t="s">
+        <v>76</v>
+      </c>
+      <c r="AT16" t="s">
         <v>79</v>
       </c>
-      <c r="AP2" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="AQ2" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="AR2" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="AS2" t="s">
-        <v>83</v>
-      </c>
-      <c r="AT2" t="s">
-        <v>86</v>
-      </c>
-      <c r="AU2" t="s">
-        <v>87</v>
-      </c>
-      <c r="AV2" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="AW2" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="AX2" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="AY2" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="AZ2" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="BA2" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="BB2" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="BC2" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="BD2" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="BE2" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="BF2" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="BG2" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="BH2" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="BI2" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="BJ2" s="1" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="3" spans="1:62" x14ac:dyDescent="0.25">
-      <c r="S3" s="1"/>
+      <c r="AU16" t="s">
+        <v>80</v>
+      </c>
+      <c r="AV16" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="AW16" s="1" t="s">
+        <v>84</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="AP2" r:id="rId1" xr:uid="{15FDB767-4FC8-4922-8149-ACFD636428CA}"/>
+    <hyperlink ref="AP8" r:id="rId1" xr:uid="{01E094B1-7362-4107-AE1C-4F7C28A986BF}"/>
+    <hyperlink ref="AP15" r:id="rId2" xr:uid="{15FDB767-4FC8-4922-8149-ACFD636428CA}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>